<commit_message>
feat: nine roles show Applied
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/career/job-tracker.xlsx
+++ b/public/career/job-tracker.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Job tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job tracker'!$A$4:$G$27</definedName>
@@ -582,7 +582,7 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -849,7 +849,7 @@
       <c r="E13" s="11" t="n"/>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -944,7 +944,7 @@
       <c r="E16" s="11" t="n"/>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -1039,7 +1039,7 @@
       <c r="E19" s="11" t="n"/>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -1164,7 +1164,7 @@
       <c r="E23" s="11" t="n"/>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">

</xml_diff>